<commit_message>
Aclarar qué herramientas usamos y cuáles no, en una sola tabla
Dos correcciones sobre el commit anterior:

- Sacar el tono de "el enunciado deja elegir, así que elegimos", que suena a
  justificar un atajo citando el reglamento. El criterio ahora se enuncia por
  lo que es: aplicamos la herramienta cuando producía evidencia sobre esta
  empresa, y la dejamos afuera cuando devolvía casilleros vacíos o cuando su
  resultado pertenece a una etapa posterior.
- No quedaba claro cuáles se usaron y cuáles no. herramientas.md ahora abre
  con una tabla única de 16 filas con tres columnas —herramienta, si la usamos
  y por qué— más una segunda tabla de qué se usó en cada sección. Eso se
  replica en la planilla, en el anexo II del informe y en los dos artifacts.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Material Campus/Proyecto Final/Proyecto/Entrega/TP Final Parte 1 - Dulxelitos - Planilla.xlsx
+++ b/Material Campus/Proyecto Final/Proyecto/Entrega/TP Final Parte 1 - Dulxelitos - Planilla.xlsx
@@ -130,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -196,6 +196,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2228,9 +2231,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -2254,12 +2257,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Autor u origen</t>
+          <t>¿La usamos?</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Para qué la usamos</t>
+          <t>Por qué</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -2279,7 +2282,11 @@
           <t>No aplica</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Relevamiento descriptivo según la estructura del enunciado</t>
@@ -2304,7 +2311,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Adaptado de PESTEL</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2331,7 +2338,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Porter (1979, 1980)</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -2358,7 +2365,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Porter (1985)</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2385,7 +2392,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Planeamiento clásico</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -2412,7 +2419,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Osterwalder y Pigneur (2010)</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -2439,7 +2446,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Enfoque bimodal de la materia</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -2466,7 +2473,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Porter (1980)</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -2493,7 +2500,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Osterwalder y otros (2014)</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -2520,7 +2527,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Cátedra</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -2547,7 +2554,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Fórmula de tres componentes</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -2564,125 +2571,153 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Herramientas que dejamos afuera y por qué</t>
+          <t>Las que quedaron afuera</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>PESTEL completo</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="24" t="n"/>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Cuatro de sus seis dimensiones volvían vacías en este caso. La guía de la cátedra advierte contra listar factores sin impacto real: usa 'FODA + factores clave', no un PESTEL</t>
         </is>
       </c>
-      <c r="C17" s="24" t="n"/>
-      <c r="D17" s="24" t="n"/>
       <c r="E17" s="24" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>FODA cruzado</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="24" t="n"/>
+      <c r="C18" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Su producto son iniciativas y esta entrega es diagnóstico. El FODA simple sí está, que es la forma que usa la guía de la cátedra</t>
         </is>
       </c>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="24" t="n"/>
       <c r="E18" s="24" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Hipótesis de Oportunidad Tecnológica</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Es una propuesta de solución (To-Be) y este trabajo es diagnóstico del estado actual</t>
         </is>
       </c>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
       <c r="E19" s="24" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>BMC en versión To-Be</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="24" t="n"/>
+      <c r="C20" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>El enunciado pide el modelo actual, no el propuesto</t>
         </is>
       </c>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
       <c r="E20" s="24" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Balanced Scorecard y OKR</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="24" t="n"/>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Corresponden al Hito 3</t>
         </is>
       </c>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="24" t="n"/>
       <c r="E21" s="24" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Design Thinking</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="24" t="n"/>
+      <c r="C22" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Apunta a idear soluciones, que todavía no toca</t>
         </is>
       </c>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="24" t="n"/>
       <c r="E22" s="24" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Plantilla del problema gerencial</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="24" t="n"/>
+      <c r="C23" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Es para la sección 6, que se entrega aparte</t>
         </is>
       </c>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="24" t="n"/>
       <c r="E23" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D23:E23"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D21:E21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>